<commit_message>
Playground learning only 8 horizon, menyesuaikan dataset awal yang seharusnya dimiliki
</commit_message>
<xml_diff>
--- a/wfcv_predictions.xlsx
+++ b/wfcv_predictions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="MU-250-40Kg" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="MU-302-50Kg" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MU-380-40KG" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="MU-480-Combined" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MU-250-40Kg" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MU-302-50Kg" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MU-380-40KG" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MU-480-Combined" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -530,6 +530,21 @@
           <t>Prophet_Step3</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step1</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step2</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step3</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -562,10 +577,10 @@
         <v>50409</v>
       </c>
       <c r="H2" t="n">
-        <v>50489.21751551224</v>
+        <v>50489.21751551223</v>
       </c>
       <c r="I2" t="n">
-        <v>42521.16223773449</v>
+        <v>42521.16223773448</v>
       </c>
       <c r="J2" t="n">
         <v>52915.00946284268</v>
@@ -580,13 +595,13 @@
         <v>50406.63671875</v>
       </c>
       <c r="N2" t="n">
-        <v>44015.6434886885</v>
+        <v>44015.64348868855</v>
       </c>
       <c r="O2" t="n">
-        <v>45155.19119120954</v>
+        <v>45155.19119120974</v>
       </c>
       <c r="P2" t="n">
-        <v>59091.51589704474</v>
+        <v>59091.51589704488</v>
       </c>
       <c r="Q2" t="n">
         <v>52226.44736842105</v>
@@ -598,13 +613,22 @@
         <v>52226.44736842105</v>
       </c>
       <c r="T2" t="n">
-        <v>48613.27098899829</v>
+        <v>48613.27098899803</v>
       </c>
       <c r="U2" t="n">
-        <v>24279.81460045306</v>
+        <v>24279.8146004529</v>
       </c>
       <c r="V2" t="n">
-        <v>62249.92422032052</v>
+        <v>62249.92422032026</v>
+      </c>
+      <c r="W2" t="n">
+        <v>40641</v>
+      </c>
+      <c r="X2" t="n">
+        <v>40641</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>40641</v>
       </c>
     </row>
     <row r="3">
@@ -656,13 +680,13 @@
         <v>46103.375</v>
       </c>
       <c r="N3" t="n">
-        <v>32915.79253438687</v>
+        <v>32915.79253438639</v>
       </c>
       <c r="O3" t="n">
-        <v>54992.92528854259</v>
+        <v>54992.92528854255</v>
       </c>
       <c r="P3" t="n">
-        <v>51232.30908214405</v>
+        <v>51232.30908214415</v>
       </c>
       <c r="Q3" t="n">
         <v>51439.10256410256</v>
@@ -674,13 +698,22 @@
         <v>51439.10256410256</v>
       </c>
       <c r="T3" t="n">
-        <v>-7186.767896528214</v>
+        <v>-7186.767896528076</v>
       </c>
       <c r="U3" t="n">
-        <v>6429.411454822999</v>
+        <v>6429.411454822861</v>
       </c>
       <c r="V3" t="n">
-        <v>-723.1662790660957</v>
+        <v>-723.1662790660994</v>
+      </c>
+      <c r="W3" t="n">
+        <v>21520</v>
+      </c>
+      <c r="X3" t="n">
+        <v>21520</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>21520</v>
       </c>
     </row>
     <row r="4">
@@ -714,13 +747,13 @@
         <v>52492</v>
       </c>
       <c r="H4" t="n">
-        <v>51826.82087103173</v>
+        <v>51826.82087103174</v>
       </c>
       <c r="I4" t="n">
-        <v>52130.98990602452</v>
+        <v>52130.98990602453</v>
       </c>
       <c r="J4" t="n">
-        <v>52942.04611435786</v>
+        <v>52942.04611435787</v>
       </c>
       <c r="K4" t="n">
         <v>48276.60546875</v>
@@ -732,13 +765,13 @@
         <v>49646.76953125</v>
       </c>
       <c r="N4" t="n">
-        <v>52815.96144392241</v>
+        <v>52815.96144392222</v>
       </c>
       <c r="O4" t="n">
-        <v>50555.89633137756</v>
+        <v>50555.89633137752</v>
       </c>
       <c r="P4" t="n">
-        <v>54471.36741932661</v>
+        <v>54471.36741932672</v>
       </c>
       <c r="Q4" t="n">
         <v>47740.91773307796</v>
@@ -750,13 +783,22 @@
         <v>49618.5770626068</v>
       </c>
       <c r="T4" t="n">
-        <v>52948.90786407243</v>
+        <v>52948.90786407224</v>
       </c>
       <c r="U4" t="n">
-        <v>50668.74657510391</v>
+        <v>50668.7465751037</v>
       </c>
       <c r="V4" t="n">
-        <v>41507.76441358356</v>
+        <v>41507.76441358327</v>
+      </c>
+      <c r="W4" t="n">
+        <v>28407</v>
+      </c>
+      <c r="X4" t="n">
+        <v>28407</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>28407</v>
       </c>
     </row>
     <row r="5">
@@ -793,10 +835,10 @@
         <v>50417.40760722613</v>
       </c>
       <c r="I5" t="n">
-        <v>51867.58388247866</v>
+        <v>51867.58388247864</v>
       </c>
       <c r="J5" t="n">
-        <v>52825.56793803422</v>
+        <v>52825.5679380342</v>
       </c>
       <c r="K5" t="n">
         <v>47165.35546875</v>
@@ -808,13 +850,13 @@
         <v>45742.6484375</v>
       </c>
       <c r="N5" t="n">
-        <v>49238.71638730518</v>
+        <v>49238.71638730521</v>
       </c>
       <c r="O5" t="n">
-        <v>53655.93214827742</v>
+        <v>53655.93214827761</v>
       </c>
       <c r="P5" t="n">
-        <v>57888.23433731938</v>
+        <v>57888.23433731963</v>
       </c>
       <c r="Q5" t="n">
         <v>44675.00443147335</v>
@@ -829,10 +871,19 @@
         <v>47867.62307118031</v>
       </c>
       <c r="U5" t="n">
-        <v>39247.67099800456</v>
+        <v>39247.67099800461</v>
       </c>
       <c r="V5" t="n">
-        <v>44869.71242929884</v>
+        <v>44869.7124292989</v>
+      </c>
+      <c r="W5" t="n">
+        <v>50409</v>
+      </c>
+      <c r="X5" t="n">
+        <v>50409</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>50409</v>
       </c>
     </row>
     <row r="6">
@@ -866,13 +917,13 @@
         <v>47133</v>
       </c>
       <c r="H6" t="n">
-        <v>51031.28851208512</v>
+        <v>51031.28851208511</v>
       </c>
       <c r="I6" t="n">
-        <v>50508.96789442502</v>
+        <v>50508.96789442501</v>
       </c>
       <c r="J6" t="n">
-        <v>51022.21222775835</v>
+        <v>51022.21222775834</v>
       </c>
       <c r="K6" t="n">
         <v>53341.34765625</v>
@@ -884,13 +935,13 @@
         <v>56231.34765625</v>
       </c>
       <c r="N6" t="n">
-        <v>52007.80950281813</v>
+        <v>52007.80950281792</v>
       </c>
       <c r="O6" t="n">
-        <v>57022.4967337124</v>
+        <v>57022.4967337122</v>
       </c>
       <c r="P6" t="n">
-        <v>57629.34500592703</v>
+        <v>57629.34500592681</v>
       </c>
       <c r="Q6" t="n">
         <v>45258.10968039101</v>
@@ -902,13 +953,22 @@
         <v>40426.9142611476</v>
       </c>
       <c r="T6" t="n">
-        <v>38765.62671043073</v>
+        <v>38765.62671043081</v>
       </c>
       <c r="U6" t="n">
-        <v>43495.24172693788</v>
+        <v>43495.24172693781</v>
       </c>
       <c r="V6" t="n">
-        <v>43376.12238574785</v>
+        <v>43376.12238574776</v>
+      </c>
+      <c r="W6" t="n">
+        <v>46394</v>
+      </c>
+      <c r="X6" t="n">
+        <v>46394</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>46394</v>
       </c>
     </row>
     <row r="7">
@@ -942,10 +1002,10 @@
         <v>50209</v>
       </c>
       <c r="H7" t="n">
-        <v>51086.98276401377</v>
+        <v>51086.98276401375</v>
       </c>
       <c r="I7" t="n">
-        <v>50909.32688901376</v>
+        <v>50909.32688901375</v>
       </c>
       <c r="J7" t="n">
         <v>50834.06769853758</v>
@@ -960,13 +1020,13 @@
         <v>48251.49609375</v>
       </c>
       <c r="N7" t="n">
-        <v>57139.42467040572</v>
+        <v>57139.42467040586</v>
       </c>
       <c r="O7" t="n">
-        <v>57649.04272444578</v>
+        <v>57649.04272444598</v>
       </c>
       <c r="P7" t="n">
-        <v>63725.39201813658</v>
+        <v>63725.39201813667</v>
       </c>
       <c r="Q7" t="n">
         <v>51553.26262863745</v>
@@ -978,13 +1038,22 @@
         <v>41280.87000420186</v>
       </c>
       <c r="T7" t="n">
-        <v>53939.91565221758</v>
+        <v>53939.91565221764</v>
       </c>
       <c r="U7" t="n">
-        <v>54164.58730690851</v>
+        <v>54164.58730690849</v>
       </c>
       <c r="V7" t="n">
-        <v>50759.93478864031</v>
+        <v>50759.93478864019</v>
+      </c>
+      <c r="W7" t="n">
+        <v>52492</v>
+      </c>
+      <c r="X7" t="n">
+        <v>52492</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>52492</v>
       </c>
     </row>
     <row r="8">
@@ -1018,13 +1087,13 @@
         <v>57982</v>
       </c>
       <c r="H8" t="n">
-        <v>49040.62051151624</v>
+        <v>49040.62051151625</v>
       </c>
       <c r="I8" t="n">
-        <v>48569.75401146075</v>
+        <v>48569.75401146077</v>
       </c>
       <c r="J8" t="n">
-        <v>50290.46640470643</v>
+        <v>50290.46640470641</v>
       </c>
       <c r="K8" t="n">
         <v>54142.3046875</v>
@@ -1036,13 +1105,13 @@
         <v>56951.8671875</v>
       </c>
       <c r="N8" t="n">
-        <v>52670.05534720033</v>
+        <v>52670.05534720037</v>
       </c>
       <c r="O8" t="n">
-        <v>61572.09470127478</v>
+        <v>61572.09470127489</v>
       </c>
       <c r="P8" t="n">
-        <v>50836.01248948614</v>
+        <v>50836.01248948611</v>
       </c>
       <c r="Q8" t="n">
         <v>45106.08377753541</v>
@@ -1054,13 +1123,22 @@
         <v>42096.93952878902</v>
       </c>
       <c r="T8" t="n">
-        <v>49096.34297529873</v>
+        <v>49096.34297529879</v>
       </c>
       <c r="U8" t="n">
-        <v>44672.54244660228</v>
+        <v>44672.54244660241</v>
       </c>
       <c r="V8" t="n">
-        <v>38777.50004867914</v>
+        <v>38777.50004867939</v>
+      </c>
+      <c r="W8" t="n">
+        <v>42764</v>
+      </c>
+      <c r="X8" t="n">
+        <v>42764</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>42764</v>
       </c>
     </row>
     <row r="9">
@@ -1112,13 +1190,13 @@
         <v>53242.14453125</v>
       </c>
       <c r="N9" t="n">
-        <v>59805.74113840394</v>
+        <v>59805.74113840386</v>
       </c>
       <c r="O9" t="n">
         <v>50242.69541822607</v>
       </c>
       <c r="P9" t="n">
-        <v>49129.66842833375</v>
+        <v>49129.66842833372</v>
       </c>
       <c r="Q9" t="n">
         <v>50949.52460073888</v>
@@ -1130,241 +1208,22 @@
         <v>46138.3135595171</v>
       </c>
       <c r="T9" t="n">
-        <v>43537.10829895572</v>
+        <v>43537.10829895597</v>
       </c>
       <c r="U9" t="n">
-        <v>37101.7191245709</v>
+        <v>37101.71912457116</v>
       </c>
       <c r="V9" t="n">
-        <v>37318.5204419964</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>H9</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>57982</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>60667</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>28735</v>
-      </c>
-      <c r="H10" t="n">
-        <v>49418.67935270288</v>
-      </c>
-      <c r="I10" t="n">
-        <v>49474.84010270287</v>
-      </c>
-      <c r="J10" t="n">
-        <v>46855.37079972809</v>
-      </c>
-      <c r="K10" t="n">
-        <v>53293.1875</v>
-      </c>
-      <c r="L10" t="n">
-        <v>51673.77734375</v>
-      </c>
-      <c r="M10" t="n">
-        <v>41706.7421875</v>
-      </c>
-      <c r="N10" t="n">
-        <v>47467.46940636075</v>
-      </c>
-      <c r="O10" t="n">
-        <v>47413.06635981649</v>
-      </c>
-      <c r="P10" t="n">
-        <v>47582.78336491378</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>44023.77577504936</v>
-      </c>
-      <c r="R10" t="n">
-        <v>45319.49752238245</v>
-      </c>
-      <c r="S10" t="n">
-        <v>31958.74307340965</v>
-      </c>
-      <c r="T10" t="n">
-        <v>40280.24750288138</v>
-      </c>
-      <c r="U10" t="n">
-        <v>41383.57809425767</v>
-      </c>
-      <c r="V10" t="n">
-        <v>621114.1903086904</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>H10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>60667</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>28735</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>25687</v>
-      </c>
-      <c r="H11" t="n">
-        <v>56803.99372150076</v>
-      </c>
-      <c r="I11" t="n">
-        <v>53167.2745297619</v>
-      </c>
-      <c r="J11" t="n">
-        <v>48182.17586525978</v>
-      </c>
-      <c r="K11" t="n">
-        <v>60462.734375</v>
-      </c>
-      <c r="L11" t="n">
-        <v>59249.1328125</v>
-      </c>
-      <c r="M11" t="n">
-        <v>55487.44140625</v>
-      </c>
-      <c r="N11" t="n">
-        <v>52480.37852023693</v>
-      </c>
-      <c r="O11" t="n">
-        <v>47073.38596877269</v>
-      </c>
-      <c r="P11" t="n">
-        <v>51977.92842170754</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>62411.35664202193</v>
-      </c>
-      <c r="R11" t="n">
-        <v>49127.82846422889</v>
-      </c>
-      <c r="S11" t="n">
-        <v>48783.20410974354</v>
-      </c>
-      <c r="T11" t="n">
-        <v>50804.84822174135</v>
-      </c>
-      <c r="U11" t="n">
-        <v>592654.4581616096</v>
-      </c>
-      <c r="V11" t="n">
-        <v>836682.753523075</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>H11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>28735</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>25687</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>10840</v>
-      </c>
-      <c r="H12" t="n">
-        <v>55022.95906998555</v>
-      </c>
-      <c r="I12" t="n">
-        <v>53235.66689574313</v>
-      </c>
-      <c r="J12" t="n">
-        <v>47141.28166414142</v>
-      </c>
-      <c r="K12" t="n">
-        <v>58713.1640625</v>
-      </c>
-      <c r="L12" t="n">
-        <v>55584.0078125</v>
-      </c>
-      <c r="M12" t="n">
-        <v>50830.3671875</v>
-      </c>
-      <c r="N12" t="n">
-        <v>47839.3170323433</v>
-      </c>
-      <c r="O12" t="n">
-        <v>51011.90246785057</v>
-      </c>
-      <c r="P12" t="n">
-        <v>52465.65820670298</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>52601.90855369313</v>
-      </c>
-      <c r="R12" t="n">
-        <v>41551.47257399447</v>
-      </c>
-      <c r="S12" t="n">
-        <v>52711.76939482008</v>
-      </c>
-      <c r="T12" t="n">
-        <v>591624.2592958629</v>
-      </c>
-      <c r="U12" t="n">
-        <v>915659.8699990249</v>
-      </c>
-      <c r="V12" t="n">
-        <v>781557.8108593236</v>
+        <v>37318.52044199691</v>
+      </c>
+      <c r="W9" t="n">
+        <v>47133</v>
+      </c>
+      <c r="X9" t="n">
+        <v>47133</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>47133</v>
       </c>
     </row>
   </sheetData>
@@ -1378,7 +1237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1492,6 +1351,21 @@
           <t>Prophet_Step3</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step1</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step2</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step3</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1542,13 +1416,13 @@
         <v>212149.875</v>
       </c>
       <c r="N2" t="n">
-        <v>167519.7378668202</v>
+        <v>167519.7378668197</v>
       </c>
       <c r="O2" t="n">
-        <v>22313.80817947758</v>
+        <v>22313.80817947607</v>
       </c>
       <c r="P2" t="n">
-        <v>297790.638208057</v>
+        <v>297790.6382080683</v>
       </c>
       <c r="Q2" t="n">
         <v>306718.3157894737</v>
@@ -1563,10 +1437,19 @@
         <v>590759.205376266</v>
       </c>
       <c r="U2" t="n">
-        <v>274571.707887387</v>
+        <v>274571.7078873841</v>
       </c>
       <c r="V2" t="n">
-        <v>321371.2344942054</v>
+        <v>321371.2344942087</v>
+      </c>
+      <c r="W2" t="n">
+        <v>238596.8817111391</v>
+      </c>
+      <c r="X2" t="n">
+        <v>235898.4385939329</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>237022.6825714436</v>
       </c>
     </row>
     <row r="3">
@@ -1618,13 +1501,13 @@
         <v>206412.34375</v>
       </c>
       <c r="N3" t="n">
-        <v>13056.72573106119</v>
+        <v>13056.72573105997</v>
       </c>
       <c r="O3" t="n">
-        <v>430758.7831108036</v>
+        <v>430758.7831108358</v>
       </c>
       <c r="P3" t="n">
-        <v>234386.5099578347</v>
+        <v>234386.5099578592</v>
       </c>
       <c r="Q3" t="n">
         <v>303084.8974358974</v>
@@ -1636,13 +1519,22 @@
         <v>303084.8974358974</v>
       </c>
       <c r="T3" t="n">
-        <v>-31251.32181148964</v>
+        <v>-31251.32181149005</v>
       </c>
       <c r="U3" t="n">
-        <v>-87290.91944105973</v>
+        <v>-87290.91944105734</v>
       </c>
       <c r="V3" t="n">
-        <v>-126787.0978414504</v>
+        <v>-126787.0978414516</v>
+      </c>
+      <c r="W3" t="n">
+        <v>192749.8557263461</v>
+      </c>
+      <c r="X3" t="n">
+        <v>181286.8913844754</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>186024.5959104874</v>
       </c>
     </row>
     <row r="4">
@@ -1697,10 +1589,10 @@
         <v>193014.4347739056</v>
       </c>
       <c r="O4" t="n">
-        <v>173223.4526080143</v>
+        <v>173223.452608014</v>
       </c>
       <c r="P4" t="n">
-        <v>223790.431874974</v>
+        <v>223790.4318749746</v>
       </c>
       <c r="Q4" t="n">
         <v>291248.5011633298</v>
@@ -1715,10 +1607,19 @@
         <v>243525.8164941688</v>
       </c>
       <c r="U4" t="n">
-        <v>305296.3332695057</v>
+        <v>305296.3332695063</v>
       </c>
       <c r="V4" t="n">
-        <v>352306.7493926775</v>
+        <v>352306.7493926772</v>
+      </c>
+      <c r="W4" t="n">
+        <v>171290.0629686548</v>
+      </c>
+      <c r="X4" t="n">
+        <v>173078.1197373045</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>172344.9867007727</v>
       </c>
     </row>
     <row r="5">
@@ -1758,7 +1659,7 @@
         <v>329411.5434759961</v>
       </c>
       <c r="J5" t="n">
-        <v>342991.8377292014</v>
+        <v>342991.8377292013</v>
       </c>
       <c r="K5" t="n">
         <v>329546.5625</v>
@@ -1773,10 +1674,10 @@
         <v>295943.4321392876</v>
       </c>
       <c r="O5" t="n">
-        <v>384543.2686801426</v>
+        <v>384543.2686801428</v>
       </c>
       <c r="P5" t="n">
-        <v>408568.965400014</v>
+        <v>408568.9654000142</v>
       </c>
       <c r="Q5" t="n">
         <v>372140.1444527204</v>
@@ -1788,13 +1689,22 @@
         <v>380783.2872217199</v>
       </c>
       <c r="T5" t="n">
-        <v>379617.413902332</v>
+        <v>379617.4139023311</v>
       </c>
       <c r="U5" t="n">
-        <v>430016.1503980561</v>
+        <v>430016.1503980567</v>
       </c>
       <c r="V5" t="n">
         <v>450674.7418690737</v>
+      </c>
+      <c r="W5" t="n">
+        <v>261644.7891016562</v>
+      </c>
+      <c r="X5" t="n">
+        <v>285425.6145753978</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>275783.0694916663</v>
       </c>
     </row>
     <row r="6">
@@ -1834,7 +1744,7 @@
         <v>315014.9852186148</v>
       </c>
       <c r="J6" t="n">
-        <v>318053.2991412337</v>
+        <v>318053.2991412338</v>
       </c>
       <c r="K6" t="n">
         <v>316858.4375</v>
@@ -1846,13 +1756,13 @@
         <v>341857.4375</v>
       </c>
       <c r="N6" t="n">
-        <v>363112.3684733788</v>
+        <v>363112.3684733793</v>
       </c>
       <c r="O6" t="n">
-        <v>383283.6911799797</v>
+        <v>383283.6911799805</v>
       </c>
       <c r="P6" t="n">
-        <v>417306.2338371794</v>
+        <v>417306.2338371802</v>
       </c>
       <c r="Q6" t="n">
         <v>339174.1203532174</v>
@@ -1864,13 +1774,22 @@
         <v>429811.8985696202</v>
       </c>
       <c r="T6" t="n">
-        <v>368463.171793311</v>
+        <v>368463.1717933117</v>
       </c>
       <c r="U6" t="n">
-        <v>386919.9245057401</v>
+        <v>386919.9245057392</v>
       </c>
       <c r="V6" t="n">
-        <v>393877.4646927002</v>
+        <v>393877.4646927004</v>
+      </c>
+      <c r="W6" t="n">
+        <v>285435.4586218619</v>
+      </c>
+      <c r="X6" t="n">
+        <v>275796.0580411998</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>279704.5361904003</v>
       </c>
     </row>
     <row r="7">
@@ -1922,13 +1841,13 @@
         <v>378073.5</v>
       </c>
       <c r="N7" t="n">
-        <v>344119.407046641</v>
+        <v>344119.4070466409</v>
       </c>
       <c r="O7" t="n">
-        <v>360991.6266551559</v>
+        <v>360991.6266551554</v>
       </c>
       <c r="P7" t="n">
-        <v>418584.1003417687</v>
+        <v>418584.1003417679</v>
       </c>
       <c r="Q7" t="n">
         <v>384039.1623128151</v>
@@ -1940,13 +1859,22 @@
         <v>424615.8884621104</v>
       </c>
       <c r="T7" t="n">
-        <v>341820.7580158682</v>
+        <v>341820.7580158694</v>
       </c>
       <c r="U7" t="n">
         <v>345635.3807038177</v>
       </c>
       <c r="V7" t="n">
-        <v>376161.3427573396</v>
+        <v>376161.3427573404</v>
+      </c>
+      <c r="W7" t="n">
+        <v>289040.7556166059</v>
+      </c>
+      <c r="X7" t="n">
+        <v>296790.7926406485</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>293620.9436214608</v>
       </c>
     </row>
     <row r="8">
@@ -1986,7 +1914,7 @@
         <v>305882.1205148324</v>
       </c>
       <c r="J8" t="n">
-        <v>311204.6121190889</v>
+        <v>311204.6121190891</v>
       </c>
       <c r="K8" t="n">
         <v>280689</v>
@@ -1998,13 +1926,13 @@
         <v>307845.875</v>
       </c>
       <c r="N8" t="n">
-        <v>313490.5347997571</v>
+        <v>313490.5347997582</v>
       </c>
       <c r="O8" t="n">
-        <v>354343.4473475526</v>
+        <v>354343.4473475544</v>
       </c>
       <c r="P8" t="n">
-        <v>342607.9216253858</v>
+        <v>342607.9216253882</v>
       </c>
       <c r="Q8" t="n">
         <v>320859.2845575609</v>
@@ -2019,10 +1947,19 @@
         <v>290959.1199705584</v>
       </c>
       <c r="U8" t="n">
-        <v>338408.9517927998</v>
+        <v>338408.951792799</v>
       </c>
       <c r="V8" t="n">
-        <v>301823.5444232739</v>
+        <v>301823.5444232723</v>
+      </c>
+      <c r="W8" t="n">
+        <v>269504.7571713164</v>
+      </c>
+      <c r="X8" t="n">
+        <v>258190.7339389604</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>262883.6349644863</v>
       </c>
     </row>
     <row r="9">
@@ -2056,7 +1993,7 @@
         <v>444902</v>
       </c>
       <c r="H9" t="n">
-        <v>305195.5849609002</v>
+        <v>305195.5849609001</v>
       </c>
       <c r="I9" t="n">
         <v>311941.980958014</v>
@@ -2074,13 +2011,13 @@
         <v>298473.84375</v>
       </c>
       <c r="N9" t="n">
-        <v>331436.1324380297</v>
+        <v>331436.13243803</v>
       </c>
       <c r="O9" t="n">
-        <v>310706.0774807418</v>
+        <v>310706.0774807419</v>
       </c>
       <c r="P9" t="n">
-        <v>319028.1072494244</v>
+        <v>319028.1072494249</v>
       </c>
       <c r="Q9" t="n">
         <v>314676.1959538058</v>
@@ -2092,241 +2029,22 @@
         <v>396639.2416637882</v>
       </c>
       <c r="T9" t="n">
-        <v>328147.7356071506</v>
+        <v>328147.7356071514</v>
       </c>
       <c r="U9" t="n">
-        <v>288613.8954443915</v>
+        <v>288613.8954443932</v>
       </c>
       <c r="V9" t="n">
-        <v>261838.6190625005</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>H9</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>411634</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>444902</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>243151</v>
-      </c>
-      <c r="H10" t="n">
-        <v>315980.8894013347</v>
-      </c>
-      <c r="I10" t="n">
-        <v>326858.2072267316</v>
-      </c>
-      <c r="J10" t="n">
-        <v>271246.9093531747</v>
-      </c>
-      <c r="K10" t="n">
-        <v>328498.4375</v>
-      </c>
-      <c r="L10" t="n">
-        <v>336913.9375</v>
-      </c>
-      <c r="M10" t="n">
-        <v>238203.0625</v>
-      </c>
-      <c r="N10" t="n">
-        <v>300459.0957882533</v>
-      </c>
-      <c r="O10" t="n">
-        <v>304506.0847405666</v>
-      </c>
-      <c r="P10" t="n">
-        <v>280881.2316732626</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>331685.085606301</v>
-      </c>
-      <c r="R10" t="n">
-        <v>382462.5559961111</v>
-      </c>
-      <c r="S10" t="n">
-        <v>295284.80880972</v>
-      </c>
-      <c r="T10" t="n">
-        <v>280245.6653889666</v>
-      </c>
-      <c r="U10" t="n">
-        <v>250758.9142536277</v>
-      </c>
-      <c r="V10" t="n">
-        <v>4182741.67668245</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>H10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>444902</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>243151</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>243453</v>
-      </c>
-      <c r="H11" t="n">
-        <v>376487.947853355</v>
-      </c>
-      <c r="I11" t="n">
-        <v>370287.5881228356</v>
-      </c>
-      <c r="J11" t="n">
-        <v>362737.6419990981</v>
-      </c>
-      <c r="K11" t="n">
-        <v>397721.75</v>
-      </c>
-      <c r="L11" t="n">
-        <v>372759.28125</v>
-      </c>
-      <c r="M11" t="n">
-        <v>332271.15625</v>
-      </c>
-      <c r="N11" t="n">
-        <v>401427.4511303457</v>
-      </c>
-      <c r="O11" t="n">
-        <v>317774.8761775802</v>
-      </c>
-      <c r="P11" t="n">
-        <v>295274.1086980728</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>388734.6886307122</v>
-      </c>
-      <c r="R11" t="n">
-        <v>307466.8482047298</v>
-      </c>
-      <c r="S11" t="n">
-        <v>299409.0679513096</v>
-      </c>
-      <c r="T11" t="n">
-        <v>343907.2730929527</v>
-      </c>
-      <c r="U11" t="n">
-        <v>3573242.024841727</v>
-      </c>
-      <c r="V11" t="n">
-        <v>5105523.631079276</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>H11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>243151</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>243453</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>99784</v>
-      </c>
-      <c r="H12" t="n">
-        <v>381706.7627017288</v>
-      </c>
-      <c r="I12" t="n">
-        <v>366298.0216574675</v>
-      </c>
-      <c r="J12" t="n">
-        <v>339351.8510443724</v>
-      </c>
-      <c r="K12" t="n">
-        <v>373040.875</v>
-      </c>
-      <c r="L12" t="n">
-        <v>292869.0625</v>
-      </c>
-      <c r="M12" t="n">
-        <v>302738.3125</v>
-      </c>
-      <c r="N12" t="n">
-        <v>323460.8148470639</v>
-      </c>
-      <c r="O12" t="n">
-        <v>304068.82353864</v>
-      </c>
-      <c r="P12" t="n">
-        <v>254761.9834157388</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>307193.4221387458</v>
-      </c>
-      <c r="R12" t="n">
-        <v>298785.3120406053</v>
-      </c>
-      <c r="S12" t="n">
-        <v>298785.3120406053</v>
-      </c>
-      <c r="T12" t="n">
-        <v>2993003.148947143</v>
-      </c>
-      <c r="U12" t="n">
-        <v>4366777.61444292</v>
-      </c>
-      <c r="V12" t="n">
-        <v>3986391.730221227</v>
+        <v>261838.6190625021</v>
+      </c>
+      <c r="W9" t="n">
+        <v>263601.5989566527</v>
+      </c>
+      <c r="X9" t="n">
+        <v>269951.9356752779</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>267307.626432177</v>
       </c>
     </row>
   </sheetData>
@@ -2340,7 +2058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2454,6 +2172,21 @@
           <t>Prophet_Step3</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step1</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step2</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step3</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2486,7 +2219,7 @@
         <v>468272</v>
       </c>
       <c r="H2" t="n">
-        <v>403181.8229655484</v>
+        <v>403181.8229655485</v>
       </c>
       <c r="I2" t="n">
         <v>282677.6101998556</v>
@@ -2504,13 +2237,13 @@
         <v>430050.90625</v>
       </c>
       <c r="N2" t="n">
-        <v>339650.6051016279</v>
+        <v>339650.6051016269</v>
       </c>
       <c r="O2" t="n">
-        <v>316432.7698987697</v>
+        <v>316432.7698987699</v>
       </c>
       <c r="P2" t="n">
-        <v>429744.9360228592</v>
+        <v>429744.9360228601</v>
       </c>
       <c r="Q2" t="n">
         <v>415245.6315789474</v>
@@ -2522,13 +2255,22 @@
         <v>415245.6315789474</v>
       </c>
       <c r="T2" t="n">
-        <v>440618.1959339075</v>
+        <v>440618.1959339071</v>
       </c>
       <c r="U2" t="n">
-        <v>240277.734751242</v>
+        <v>240277.7347512424</v>
       </c>
       <c r="V2" t="n">
-        <v>365616.9645074117</v>
+        <v>365616.9645074119</v>
+      </c>
+      <c r="W2" t="n">
+        <v>382001.9825937494</v>
+      </c>
+      <c r="X2" t="n">
+        <v>340314.1673702149</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>389475.3601581438</v>
       </c>
     </row>
     <row r="3">
@@ -2568,7 +2310,7 @@
         <v>456448.5079316378</v>
       </c>
       <c r="J3" t="n">
-        <v>433984.6190546539</v>
+        <v>433984.6190546538</v>
       </c>
       <c r="K3" t="n">
         <v>247612.125</v>
@@ -2580,13 +2322,13 @@
         <v>446862.125</v>
       </c>
       <c r="N3" t="n">
-        <v>318584.9185018823</v>
+        <v>318584.9185018812</v>
       </c>
       <c r="O3" t="n">
-        <v>431700.990743077</v>
+        <v>431700.990743076</v>
       </c>
       <c r="P3" t="n">
-        <v>461652.8476056533</v>
+        <v>461652.8476056528</v>
       </c>
       <c r="Q3" t="n">
         <v>412661.3846153846</v>
@@ -2598,13 +2340,22 @@
         <v>412661.3846153846</v>
       </c>
       <c r="T3" t="n">
-        <v>313378.1752520846</v>
+        <v>313378.1752520842</v>
       </c>
       <c r="U3" t="n">
         <v>378515.8813180951</v>
       </c>
       <c r="V3" t="n">
-        <v>505829.4694249847</v>
+        <v>505829.4694249856</v>
+      </c>
+      <c r="W3" t="n">
+        <v>327804.3984971889</v>
+      </c>
+      <c r="X3" t="n">
+        <v>373878.1898449028</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>408948.9407533744</v>
       </c>
     </row>
     <row r="4">
@@ -2641,7 +2392,7 @@
         <v>455327.1629514653</v>
       </c>
       <c r="I4" t="n">
-        <v>439555.9245357143</v>
+        <v>439555.9245357144</v>
       </c>
       <c r="J4" t="n">
         <v>463772.7580149572</v>
@@ -2656,13 +2407,13 @@
         <v>509419.875</v>
       </c>
       <c r="N4" t="n">
-        <v>433148.3477064113</v>
+        <v>433148.3477064118</v>
       </c>
       <c r="O4" t="n">
-        <v>462607.6533068175</v>
+        <v>462607.6533068186</v>
       </c>
       <c r="P4" t="n">
-        <v>475095.5512955514</v>
+        <v>475095.5512955525</v>
       </c>
       <c r="Q4" t="n">
         <v>431458.2281641095</v>
@@ -2674,13 +2425,22 @@
         <v>467692.3419412993</v>
       </c>
       <c r="T4" t="n">
-        <v>387864.5678786957</v>
+        <v>387864.5678786947</v>
       </c>
       <c r="U4" t="n">
-        <v>504740.4730518823</v>
+        <v>504740.4730518828</v>
       </c>
       <c r="V4" t="n">
-        <v>421339.4319187035</v>
+        <v>421339.4319187033</v>
+      </c>
+      <c r="W4" t="n">
+        <v>370776.621187008</v>
+      </c>
+      <c r="X4" t="n">
+        <v>405762.9841461966</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>406744.7152930885</v>
       </c>
     </row>
     <row r="5">
@@ -2717,7 +2477,7 @@
         <v>437906.728916847</v>
       </c>
       <c r="I5" t="n">
-        <v>463099.97908658</v>
+        <v>463099.9790865799</v>
       </c>
       <c r="J5" t="n">
         <v>467708.8006834416</v>
@@ -2732,13 +2492,13 @@
         <v>460076.46875</v>
       </c>
       <c r="N5" t="n">
-        <v>464857.4679020488</v>
+        <v>464857.4679020508</v>
       </c>
       <c r="O5" t="n">
-        <v>473538.1465418343</v>
+        <v>473538.1465418323</v>
       </c>
       <c r="P5" t="n">
-        <v>551687.7060226565</v>
+        <v>551687.7060226592</v>
       </c>
       <c r="Q5" t="n">
         <v>453794.5595474091</v>
@@ -2750,13 +2510,22 @@
         <v>555594.1535190706</v>
       </c>
       <c r="T5" t="n">
-        <v>431932.1897633554</v>
+        <v>431932.189763356</v>
       </c>
       <c r="U5" t="n">
-        <v>477764.2213440546</v>
+        <v>477764.2213440537</v>
       </c>
       <c r="V5" t="n">
-        <v>494996.2578071995</v>
+        <v>494996.2578071997</v>
+      </c>
+      <c r="W5" t="n">
+        <v>417910.9626252678</v>
+      </c>
+      <c r="X5" t="n">
+        <v>445753.1248217066</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>531231.6111783071</v>
       </c>
     </row>
     <row r="6">
@@ -2790,7 +2559,7 @@
         <v>554969</v>
       </c>
       <c r="H6" t="n">
-        <v>461959.6079368685</v>
+        <v>461959.6079368686</v>
       </c>
       <c r="I6" t="n">
         <v>474013.769602592</v>
@@ -2808,13 +2577,13 @@
         <v>481302.15625</v>
       </c>
       <c r="N6" t="n">
-        <v>475161.1167653215</v>
+        <v>475161.1167653214</v>
       </c>
       <c r="O6" t="n">
-        <v>557282.7392489563</v>
+        <v>557282.7392489561</v>
       </c>
       <c r="P6" t="n">
-        <v>526509.6114067057</v>
+        <v>526509.6114067049</v>
       </c>
       <c r="Q6" t="n">
         <v>467976.4932590995</v>
@@ -2826,13 +2595,22 @@
         <v>538040.9861071965</v>
       </c>
       <c r="T6" t="n">
-        <v>415314.7727158376</v>
+        <v>415314.7727158375</v>
       </c>
       <c r="U6" t="n">
-        <v>530697.4906077986</v>
+        <v>530697.4906077981</v>
       </c>
       <c r="V6" t="n">
-        <v>546790.9701040295</v>
+        <v>546790.9701040296</v>
+      </c>
+      <c r="W6" t="n">
+        <v>451072.2361361859</v>
+      </c>
+      <c r="X6" t="n">
+        <v>523825.8867543603</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>485592.2631432471</v>
       </c>
     </row>
     <row r="7">
@@ -2872,7 +2650,7 @@
         <v>518374.2419494948</v>
       </c>
       <c r="J7" t="n">
-        <v>496733.380004329</v>
+        <v>496733.3800043291</v>
       </c>
       <c r="K7" t="n">
         <v>452518.09375</v>
@@ -2884,13 +2662,13 @@
         <v>527122.1875</v>
       </c>
       <c r="N7" t="n">
-        <v>555957.8355493627</v>
+        <v>555957.8355493631</v>
       </c>
       <c r="O7" t="n">
-        <v>520875.9242202161</v>
+        <v>520875.9242202164</v>
       </c>
       <c r="P7" t="n">
-        <v>443709.5813589544</v>
+        <v>443709.581358955</v>
       </c>
       <c r="Q7" t="n">
         <v>522182.9583714398</v>
@@ -2902,13 +2680,22 @@
         <v>434292.3993038851</v>
       </c>
       <c r="T7" t="n">
-        <v>483207.0037035546</v>
+        <v>483207.0037035547</v>
       </c>
       <c r="U7" t="n">
-        <v>565701.6369467746</v>
+        <v>565701.6369467743</v>
       </c>
       <c r="V7" t="n">
-        <v>490551.1522884491</v>
+        <v>490551.1522884492</v>
+      </c>
+      <c r="W7" t="n">
+        <v>534684.6988540151</v>
+      </c>
+      <c r="X7" t="n">
+        <v>490355.6041924091</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>404868.8666143786</v>
       </c>
     </row>
     <row r="8">
@@ -2942,13 +2729,13 @@
         <v>543104</v>
       </c>
       <c r="H8" t="n">
-        <v>507057.606737554</v>
+        <v>507057.6067375541</v>
       </c>
       <c r="I8" t="n">
-        <v>500471.5617357503</v>
+        <v>500471.5617357502</v>
       </c>
       <c r="J8" t="n">
-        <v>474332.5331673879</v>
+        <v>474332.5331673878</v>
       </c>
       <c r="K8" t="n">
         <v>477701.5625</v>
@@ -2960,13 +2747,13 @@
         <v>479379.90625</v>
       </c>
       <c r="N8" t="n">
-        <v>518523.7457560196</v>
+        <v>518523.7457560207</v>
       </c>
       <c r="O8" t="n">
-        <v>447243.5978859803</v>
+        <v>447243.5978859796</v>
       </c>
       <c r="P8" t="n">
-        <v>461141.3503902401</v>
+        <v>461141.3503902407</v>
       </c>
       <c r="Q8" t="n">
         <v>577652.4098391343</v>
@@ -2981,10 +2768,19 @@
         <v>561894.4924381304</v>
       </c>
       <c r="U8" t="n">
-        <v>490364.3836180858</v>
+        <v>490364.3836180851</v>
       </c>
       <c r="V8" t="n">
-        <v>489817.1566628445</v>
+        <v>489817.1566628448</v>
+      </c>
+      <c r="W8" t="n">
+        <v>483466.923683673</v>
+      </c>
+      <c r="X8" t="n">
+        <v>401855.6985318157</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>363640.7856091238</v>
       </c>
     </row>
     <row r="9">
@@ -3018,7 +2814,7 @@
         <v>593701</v>
       </c>
       <c r="H9" t="n">
-        <v>503097.5933005048</v>
+        <v>503097.5933005047</v>
       </c>
       <c r="I9" t="n">
         <v>472995.5075577197</v>
@@ -3036,13 +2832,13 @@
         <v>508093.84375</v>
       </c>
       <c r="N9" t="n">
-        <v>448767.7001387767</v>
+        <v>448767.7001387777</v>
       </c>
       <c r="O9" t="n">
-        <v>460710.1478697891</v>
+        <v>460710.1478697895</v>
       </c>
       <c r="P9" t="n">
-        <v>491237.3028005619</v>
+        <v>491237.3028005621</v>
       </c>
       <c r="Q9" t="n">
         <v>440627.8575308452</v>
@@ -3054,241 +2850,22 @@
         <v>488682.4354316772</v>
       </c>
       <c r="T9" t="n">
-        <v>496807.4432629887</v>
+        <v>496807.4432629891</v>
       </c>
       <c r="U9" t="n">
-        <v>489880.0541952213</v>
+        <v>489880.0541952203</v>
       </c>
       <c r="V9" t="n">
-        <v>469289.4676514708</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>H9</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>543104</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>593701</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>204207</v>
-      </c>
-      <c r="H10" t="n">
-        <v>472289.0989589854</v>
-      </c>
-      <c r="I10" t="n">
-        <v>509317.158578033</v>
-      </c>
-      <c r="J10" t="n">
-        <v>342139.208034632</v>
-      </c>
-      <c r="K10" t="n">
-        <v>497610.09375</v>
-      </c>
-      <c r="L10" t="n">
-        <v>506385.59375</v>
-      </c>
-      <c r="M10" t="n">
-        <v>336091.78125</v>
-      </c>
-      <c r="N10" t="n">
-        <v>439105.4698291656</v>
-      </c>
-      <c r="O10" t="n">
-        <v>489311.7868008842</v>
-      </c>
-      <c r="P10" t="n">
-        <v>230153.9329775817</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>487178.5509129612</v>
-      </c>
-      <c r="R10" t="n">
-        <v>487178.5509129612</v>
-      </c>
-      <c r="S10" t="n">
-        <v>333868.2443649733</v>
-      </c>
-      <c r="T10" t="n">
-        <v>466819.1732772405</v>
-      </c>
-      <c r="U10" t="n">
-        <v>478079.5955493556</v>
-      </c>
-      <c r="V10" t="n">
-        <v>-1126335.159215881</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>H10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>593701</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>204207</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>184105</v>
-      </c>
-      <c r="H11" t="n">
-        <v>516128.7109169582</v>
-      </c>
-      <c r="I11" t="n">
-        <v>330607.052874459</v>
-      </c>
-      <c r="J11" t="n">
-        <v>427495.4689283217</v>
-      </c>
-      <c r="K11" t="n">
-        <v>514162.59375</v>
-      </c>
-      <c r="L11" t="n">
-        <v>338381.3125</v>
-      </c>
-      <c r="M11" t="n">
-        <v>315819.1875</v>
-      </c>
-      <c r="N11" t="n">
-        <v>473044.2412662965</v>
-      </c>
-      <c r="O11" t="n">
-        <v>219169.7329334916</v>
-      </c>
-      <c r="P11" t="n">
-        <v>290885.426037775</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>482132.0910608348</v>
-      </c>
-      <c r="R11" t="n">
-        <v>332871.6051086654</v>
-      </c>
-      <c r="S11" t="n">
-        <v>352885.9681043973</v>
-      </c>
-      <c r="T11" t="n">
-        <v>441594.4179617764</v>
-      </c>
-      <c r="U11" t="n">
-        <v>-1398382.722526727</v>
-      </c>
-      <c r="V11" t="n">
-        <v>-368428.5407283364</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>H11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>204207</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>184105</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>143832</v>
-      </c>
-      <c r="H12" t="n">
-        <v>341928.509518759</v>
-      </c>
-      <c r="I12" t="n">
-        <v>443711.3496956378</v>
-      </c>
-      <c r="J12" t="n">
-        <v>340672.3810218252</v>
-      </c>
-      <c r="K12" t="n">
-        <v>358588.375</v>
-      </c>
-      <c r="L12" t="n">
-        <v>320854.8125</v>
-      </c>
-      <c r="M12" t="n">
-        <v>349025.40625</v>
-      </c>
-      <c r="N12" t="n">
-        <v>196772.2872816288</v>
-      </c>
-      <c r="O12" t="n">
-        <v>273187.3546644333</v>
-      </c>
-      <c r="P12" t="n">
-        <v>336133.2482876551</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>342711.1772480354</v>
-      </c>
-      <c r="R12" t="n">
-        <v>375661.1946030329</v>
-      </c>
-      <c r="S12" t="n">
-        <v>381908.1986774202</v>
-      </c>
-      <c r="T12" t="n">
-        <v>-1252995.803776821</v>
-      </c>
-      <c r="U12" t="n">
-        <v>-543590.3349658882</v>
-      </c>
-      <c r="V12" t="n">
-        <v>-2682993.802663302</v>
+        <v>469289.4676514717</v>
+      </c>
+      <c r="W9" t="n">
+        <v>407651.6809440249</v>
+      </c>
+      <c r="X9" t="n">
+        <v>361292.2247172176</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>372882.8053791294</v>
       </c>
     </row>
   </sheetData>
@@ -3302,7 +2879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3416,6 +2993,21 @@
           <t>Prophet_Step3</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step1</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step2</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>ARIMAX_Step3</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3466,13 +3058,13 @@
         <v>22319.96484375</v>
       </c>
       <c r="N2" t="n">
-        <v>27019.57385612314</v>
+        <v>27019.57385612302</v>
       </c>
       <c r="O2" t="n">
-        <v>27857.99105721217</v>
+        <v>27857.99105721208</v>
       </c>
       <c r="P2" t="n">
-        <v>24382.45604953514</v>
+        <v>24382.45604953506</v>
       </c>
       <c r="Q2" t="n">
         <v>18561.18421052632</v>
@@ -3487,10 +3079,19 @@
         <v>38382.67105705736</v>
       </c>
       <c r="U2" t="n">
-        <v>18551.80117878181</v>
+        <v>18551.80117878193</v>
       </c>
       <c r="V2" t="n">
-        <v>26847.58756507422</v>
+        <v>26847.58756507441</v>
+      </c>
+      <c r="W2" t="n">
+        <v>20735.51937914085</v>
+      </c>
+      <c r="X2" t="n">
+        <v>19622.23248513257</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>19139.87519537174</v>
       </c>
     </row>
     <row r="3">
@@ -3542,13 +3143,13 @@
         <v>23762.486328125</v>
       </c>
       <c r="N3" t="n">
-        <v>25599.23995604935</v>
+        <v>25599.23995604941</v>
       </c>
       <c r="O3" t="n">
-        <v>23205.07329904649</v>
+        <v>23205.07329904661</v>
       </c>
       <c r="P3" t="n">
-        <v>22916.06673155831</v>
+        <v>22916.06673155835</v>
       </c>
       <c r="Q3" t="n">
         <v>18662.87179487179</v>
@@ -3560,13 +3161,22 @@
         <v>18662.87179487179</v>
       </c>
       <c r="T3" t="n">
-        <v>17349.91024230081</v>
+        <v>17349.91024230087</v>
       </c>
       <c r="U3" t="n">
-        <v>25473.92646255292</v>
+        <v>25473.92646255299</v>
       </c>
       <c r="V3" t="n">
-        <v>26437.29984402304</v>
+        <v>26437.29984402313</v>
+      </c>
+      <c r="W3" t="n">
+        <v>20440.21746444594</v>
+      </c>
+      <c r="X3" t="n">
+        <v>19532.14506735146</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>19136.99345748525</v>
       </c>
     </row>
     <row r="4">
@@ -3618,13 +3228,13 @@
         <v>23561.708984375</v>
       </c>
       <c r="N4" t="n">
-        <v>21660.9603322794</v>
+        <v>21660.96033227898</v>
       </c>
       <c r="O4" t="n">
-        <v>22643.60075946491</v>
+        <v>22643.60075946467</v>
       </c>
       <c r="P4" t="n">
-        <v>21816.55266047882</v>
+        <v>21816.55266047861</v>
       </c>
       <c r="Q4" t="n">
         <v>18165.25005126955</v>
@@ -3636,13 +3246,22 @@
         <v>19217.74996302605</v>
       </c>
       <c r="T4" t="n">
-        <v>26947.30564685313</v>
+        <v>26947.30564685321</v>
       </c>
       <c r="U4" t="n">
-        <v>28085.03702657919</v>
+        <v>28085.03702657921</v>
       </c>
       <c r="V4" t="n">
-        <v>22340.01328691413</v>
+        <v>22340.01328691417</v>
+      </c>
+      <c r="W4" t="n">
+        <v>19245.25372554182</v>
+      </c>
+      <c r="X4" t="n">
+        <v>19000.64388725021</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>18894.31893104032</v>
       </c>
     </row>
     <row r="5">
@@ -3679,7 +3298,7 @@
         <v>22921.08865430402</v>
       </c>
       <c r="I5" t="n">
-        <v>23344.280370227</v>
+        <v>23344.28037022699</v>
       </c>
       <c r="J5" t="n">
         <v>24834.46303200965</v>
@@ -3694,13 +3313,13 @@
         <v>26199.658203125</v>
       </c>
       <c r="N5" t="n">
-        <v>23416.65914441277</v>
+        <v>23416.65914441271</v>
       </c>
       <c r="O5" t="n">
-        <v>22055.73274737781</v>
+        <v>22055.73274737761</v>
       </c>
       <c r="P5" t="n">
-        <v>22401.74087484691</v>
+        <v>22401.74087484669</v>
       </c>
       <c r="Q5" t="n">
         <v>25713.84776665547</v>
@@ -3715,10 +3334,19 @@
         <v>25765.31286922287</v>
       </c>
       <c r="U5" t="n">
-        <v>20457.30063833074</v>
+        <v>20457.30063833073</v>
       </c>
       <c r="V5" t="n">
-        <v>23233.69768652896</v>
+        <v>23233.69768652904</v>
+      </c>
+      <c r="W5" t="n">
+        <v>20994.53216229354</v>
+      </c>
+      <c r="X5" t="n">
+        <v>19844.03740828852</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>19342.93792106466</v>
       </c>
     </row>
     <row r="6">
@@ -3758,7 +3386,7 @@
         <v>25395.94589484128</v>
       </c>
       <c r="J6" t="n">
-        <v>25801.90779401155</v>
+        <v>25801.90779401156</v>
       </c>
       <c r="K6" t="n">
         <v>26555.21484375</v>
@@ -3770,13 +3398,13 @@
         <v>26531.529296875</v>
       </c>
       <c r="N6" t="n">
-        <v>22880.57464150558</v>
+        <v>22880.57464150543</v>
       </c>
       <c r="O6" t="n">
-        <v>22768.8183028726</v>
+        <v>22768.81830287238</v>
       </c>
       <c r="P6" t="n">
-        <v>23368.69218142857</v>
+        <v>23368.69218142834</v>
       </c>
       <c r="Q6" t="n">
         <v>16401.72313263551</v>
@@ -3791,10 +3419,19 @@
         <v>20591.56362554789</v>
       </c>
       <c r="U6" t="n">
-        <v>23382.05629701313</v>
+        <v>23382.05629701316</v>
       </c>
       <c r="V6" t="n">
-        <v>27709.59981564464</v>
+        <v>27709.59981564467</v>
+      </c>
+      <c r="W6" t="n">
+        <v>22193.18914193175</v>
+      </c>
+      <c r="X6" t="n">
+        <v>20475.67285676423</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>19718.29020140243</v>
       </c>
     </row>
     <row r="7">
@@ -3831,10 +3468,10 @@
         <v>24605.02146879508</v>
       </c>
       <c r="I7" t="n">
-        <v>25351.84370526695</v>
+        <v>25351.84370526694</v>
       </c>
       <c r="J7" t="n">
-        <v>24520.98230447329</v>
+        <v>24520.9823044733</v>
       </c>
       <c r="K7" t="n">
         <v>25764.72265625</v>
@@ -3846,13 +3483,13 @@
         <v>25730.97265625</v>
       </c>
       <c r="N7" t="n">
-        <v>22908.62740154944</v>
+        <v>22908.62740154961</v>
       </c>
       <c r="O7" t="n">
-        <v>23420.28218180171</v>
+        <v>23420.28218180189</v>
       </c>
       <c r="P7" t="n">
-        <v>23656.57888606753</v>
+        <v>23656.57888606784</v>
       </c>
       <c r="Q7" t="n">
         <v>23791.99903987825</v>
@@ -3864,13 +3501,22 @@
         <v>23791.99903987825</v>
       </c>
       <c r="T7" t="n">
-        <v>26483.6772104516</v>
+        <v>26483.67721045165</v>
       </c>
       <c r="U7" t="n">
-        <v>31146.41056723634</v>
+        <v>31146.41056723633</v>
       </c>
       <c r="V7" t="n">
-        <v>17985.43414741768</v>
+        <v>17985.43414741767</v>
+      </c>
+      <c r="W7" t="n">
+        <v>21000.58682865098</v>
+      </c>
+      <c r="X7" t="n">
+        <v>19973.70065885861</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>19519.06186541865</v>
       </c>
     </row>
     <row r="8">
@@ -3904,13 +3550,13 @@
         <v>31265</v>
       </c>
       <c r="H8" t="n">
-        <v>25877.74669083695</v>
+        <v>25877.74669083694</v>
       </c>
       <c r="I8" t="n">
-        <v>24780.65327651515</v>
+        <v>24780.65327651516</v>
       </c>
       <c r="J8" t="n">
-        <v>26310.52713564213</v>
+        <v>26310.52713564214</v>
       </c>
       <c r="K8" t="n">
         <v>28089.765625</v>
@@ -3922,13 +3568,13 @@
         <v>28236.943359375</v>
       </c>
       <c r="N8" t="n">
-        <v>25005.41864328671</v>
+        <v>25005.41864328685</v>
       </c>
       <c r="O8" t="n">
-        <v>24387.80360055078</v>
+        <v>24387.80360055086</v>
       </c>
       <c r="P8" t="n">
-        <v>26752.06107450637</v>
+        <v>26752.06107450621</v>
       </c>
       <c r="Q8" t="n">
         <v>25882.74085351407</v>
@@ -3947,6 +3593,15 @@
       </c>
       <c r="V8" t="n">
         <v>18911.34804960547</v>
+      </c>
+      <c r="W8" t="n">
+        <v>23132.4593997553</v>
+      </c>
+      <c r="X8" t="n">
+        <v>21059.65973782939</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>20128.98484281115</v>
       </c>
     </row>
     <row r="9">
@@ -3983,7 +3638,7 @@
         <v>24880.03996292596</v>
       </c>
       <c r="I9" t="n">
-        <v>26070.03245300533</v>
+        <v>26070.03245300532</v>
       </c>
       <c r="J9" t="n">
         <v>26290.15598871961</v>
@@ -3998,13 +3653,13 @@
         <v>29403.171875</v>
       </c>
       <c r="N9" t="n">
-        <v>25395.52626795149</v>
+        <v>25395.52626795125</v>
       </c>
       <c r="O9" t="n">
-        <v>26932.28778958239</v>
+        <v>26932.28778958254</v>
       </c>
       <c r="P9" t="n">
-        <v>28073.99562352169</v>
+        <v>28073.99562352199</v>
       </c>
       <c r="Q9" t="n">
         <v>25509.18953532243</v>
@@ -4016,241 +3671,22 @@
         <v>25724.69132460618</v>
       </c>
       <c r="T9" t="n">
-        <v>17403.53259009083</v>
+        <v>17403.53259009071</v>
       </c>
       <c r="U9" t="n">
-        <v>17999.4045733079</v>
+        <v>17999.40457330779</v>
       </c>
       <c r="V9" t="n">
         <v>20375.6627589122</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>H9</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>31265</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>34846</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>13910</v>
-      </c>
-      <c r="H10" t="n">
-        <v>26330.458505772</v>
-      </c>
-      <c r="I10" t="n">
-        <v>26343.18154545454</v>
-      </c>
-      <c r="J10" t="n">
-        <v>21776.02065079365</v>
-      </c>
-      <c r="K10" t="n">
-        <v>28440.9921875</v>
-      </c>
-      <c r="L10" t="n">
-        <v>28891.0390625</v>
-      </c>
-      <c r="M10" t="n">
-        <v>23224.7890625</v>
-      </c>
-      <c r="N10" t="n">
-        <v>26871.21081822502</v>
-      </c>
-      <c r="O10" t="n">
-        <v>28066.3846513169</v>
-      </c>
-      <c r="P10" t="n">
-        <v>15850.53430457351</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>26578.63506410913</v>
-      </c>
-      <c r="R10" t="n">
-        <v>25335.72566852138</v>
-      </c>
-      <c r="S10" t="n">
-        <v>17893.67973378346</v>
-      </c>
-      <c r="T10" t="n">
-        <v>25759.47226827441</v>
-      </c>
-      <c r="U10" t="n">
-        <v>28710.83890891517</v>
-      </c>
-      <c r="V10" t="n">
-        <v>339348.1516858765</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>H10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>34846</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>13910</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>15788</v>
-      </c>
-      <c r="H11" t="n">
-        <v>25492.79113347765</v>
-      </c>
-      <c r="I11" t="n">
-        <v>21521.36435804473</v>
-      </c>
-      <c r="J11" t="n">
-        <v>20127.75128156566</v>
-      </c>
-      <c r="K11" t="n">
-        <v>23065.97265625</v>
-      </c>
-      <c r="L11" t="n">
-        <v>22399.234375</v>
-      </c>
-      <c r="M11" t="n">
-        <v>19661.37109375</v>
-      </c>
-      <c r="N11" t="n">
-        <v>29858.97526547068</v>
-      </c>
-      <c r="O11" t="n">
-        <v>15875.72542525889</v>
-      </c>
-      <c r="P11" t="n">
-        <v>14303.34916426871</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>26994.80108916937</v>
-      </c>
-      <c r="R11" t="n">
-        <v>18650.24806504898</v>
-      </c>
-      <c r="S11" t="n">
-        <v>17373.77750542059</v>
-      </c>
-      <c r="T11" t="n">
-        <v>31619.05285309612</v>
-      </c>
-      <c r="U11" t="n">
-        <v>342184.2239583753</v>
-      </c>
-      <c r="V11" t="n">
-        <v>468717.5439120748</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>H11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>13910</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>15788</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>9568</v>
-      </c>
-      <c r="H12" t="n">
-        <v>20191.98133784271</v>
-      </c>
-      <c r="I12" t="n">
-        <v>19675.97881655844</v>
-      </c>
-      <c r="J12" t="n">
-        <v>19795.98767694805</v>
-      </c>
-      <c r="K12" t="n">
-        <v>18952.8125</v>
-      </c>
-      <c r="L12" t="n">
-        <v>17786.3359375</v>
-      </c>
-      <c r="M12" t="n">
-        <v>15202.376953125</v>
-      </c>
-      <c r="N12" t="n">
-        <v>16773.76658538989</v>
-      </c>
-      <c r="O12" t="n">
-        <v>13879.87732776346</v>
-      </c>
-      <c r="P12" t="n">
-        <v>15811.78334050314</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>19572.5356961941</v>
-      </c>
-      <c r="R12" t="n">
-        <v>18428.36188414507</v>
-      </c>
-      <c r="S12" t="n">
-        <v>18428.36188414507</v>
-      </c>
-      <c r="T12" t="n">
-        <v>364162.2046324734</v>
-      </c>
-      <c r="U12" t="n">
-        <v>489500.7508378004</v>
-      </c>
-      <c r="V12" t="n">
-        <v>402064.9730105376</v>
+      <c r="W9" t="n">
+        <v>23461.21334589524</v>
+      </c>
+      <c r="X9" t="n">
+        <v>21330.70766336601</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>20354.31214319702</v>
       </c>
     </row>
   </sheetData>

</xml_diff>